<commit_message>
Generating autogen excel code
</commit_message>
<xml_diff>
--- a/Documentation/AutoGen/AutoGenCode.xlsx
+++ b/Documentation/AutoGen/AutoGenCode.xlsx
@@ -1322,7 +1322,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="11.9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="36.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="2" width="22.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="22.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="27.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="22.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="34.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="8.61"/>
@@ -1432,8 +1432,8 @@
         <v>23</v>
       </c>
       <c r="P2" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O2," ",LOWER(F2), " _", LOWER(H2),"(", I2 ,");")</f>
-        <v>typedef LMS7002M_t* create_num _internal(LMS7002M_spi_transact_t);</v>
+        <f aca="false">CONCATENATE("typedef ",O2," ",LOWER(F2), "_", LOWER(H2),"(", I2 ,");")</f>
+        <v>typedef LMS7002M_t* create_num_internal(LMS7002M_spi_transact_t);</v>
       </c>
     </row>
     <row r="3" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1511,8 +1511,8 @@
         <v>31</v>
       </c>
       <c r="P4" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O4," ",LOWER(F4), " _", LOWER(H4),"(", I4 ,");")</f>
-        <v>typedef void one_param_lms7002m_t_num _regs(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O4," ",LOWER(F4), "_", LOWER(H4),"(", I4 ,");")</f>
+        <v>typedef void one_param_lms7002m_t_num_regs(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1563,8 +1563,8 @@
         <v>31</v>
       </c>
       <c r="P5" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O5," ",LOWER(F5), " _", LOWER(H5),"(", I5 ,");")</f>
-        <v>typedef void one_param_lms7002m_t_num _internal(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O5," ",LOWER(F5), "_", LOWER(H5),"(", I5 ,");")</f>
+        <v>typedef void one_param_lms7002m_t_num_internal(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1615,8 +1615,8 @@
         <v>31</v>
       </c>
       <c r="P6" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O6," ",LOWER(F6), " _", LOWER(H6),"(", I6 ,");")</f>
-        <v>typedef void one_param_lms7002m_t_num _regs(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O6," ",LOWER(F6), "_", LOWER(H6),"(", I6 ,");")</f>
+        <v>typedef void one_param_lms7002m_t_num_regs(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1667,8 +1667,8 @@
         <v>31</v>
       </c>
       <c r="P7" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O7," ",LOWER(F7), " _", LOWER(H7),"(", I7 ,");")</f>
-        <v>typedef void one_param_lms7002m_t_num _regs(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O7," ",LOWER(F7), "_", LOWER(H7),"(", I7 ,");")</f>
+        <v>typedef void one_param_lms7002m_t_num_regs(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1719,8 +1719,8 @@
         <v>31</v>
       </c>
       <c r="P8" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O8," ",LOWER(F8), " _", LOWER(H8),"(", I8 ,");")</f>
-        <v>typedef void one_param_lms7002m_t_num _power(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O8," ",LOWER(F8), "_", LOWER(H8),"(", I8 ,");")</f>
+        <v>typedef void one_param_lms7002m_t_num_power(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1771,8 +1771,8 @@
         <v>31</v>
       </c>
       <c r="P9" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O9," ",LOWER(F9), " _", LOWER(H9),"(", I9 ,");")</f>
-        <v>typedef void one_param_lms7002m_t_num _power(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O9," ",LOWER(F9), "_", LOWER(H9),"(", I9 ,");")</f>
+        <v>typedef void one_param_lms7002m_t_num_power(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1823,8 +1823,8 @@
         <v>31</v>
       </c>
       <c r="P10" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O10," ",LOWER(F10), " _", LOWER(H10),"(", I10 ,");")</f>
-        <v>typedef void one_param_lms7002m_t_num _loopback(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O10," ",LOWER(F10), "_", LOWER(H10),"(", I10 ,");")</f>
+        <v>typedef void one_param_lms7002m_t_num_loopback(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="11" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1852,7 +1852,10 @@
         <v>24</v>
       </c>
       <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
+      <c r="P11" s="2" t="str">
+        <f aca="false">CONCATENATE("typedef ",O11," ",LOWER(F11), "_", LOWER(H11),"(", I11 ,");")</f>
+        <v>typedef  _();</v>
+      </c>
       <c r="Q11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1903,8 +1906,8 @@
         <v>31</v>
       </c>
       <c r="P12" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O12," ",LOWER(F12), " _", LOWER(H12),"(", I12 ,");")</f>
-        <v>typedef void spi_write_num _spi(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O12," ",LOWER(F12), "_", LOWER(H12),"(", I12 ,");")</f>
+        <v>typedef void spi_write_num_spi(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="13" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1932,7 +1935,10 @@
         <v>24</v>
       </c>
       <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
+      <c r="P13" s="2" t="str">
+        <f aca="false">CONCATENATE("typedef ",O13," ",LOWER(F13), "_", LOWER(H13),"(", I13 ,");")</f>
+        <v>typedef  _();</v>
+      </c>
       <c r="Q13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1983,8 +1989,8 @@
         <v>55</v>
       </c>
       <c r="P14" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O14," ",LOWER(F14), " _", LOWER(H14),"(", I14 ,");")</f>
-        <v>typedef int spi_config_num _spi(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O14," ",LOWER(F14), "_", LOWER(H14),"(", I14 ,");")</f>
+        <v>typedef int spi_config_num_spi(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2035,8 +2041,8 @@
         <v>31</v>
       </c>
       <c r="P15" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O15," ",LOWER(F15), " _", LOWER(H15),"(", I15 ,");")</f>
-        <v>typedef void spi_config_num _spi(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O15," ",LOWER(F15), "_", LOWER(H15),"(", I15 ,");")</f>
+        <v>typedef void spi_config_num_spi(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2087,8 +2093,8 @@
         <v>31</v>
       </c>
       <c r="P16" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O16," ",LOWER(F16), " _", LOWER(H16),"(", I16 ,");")</f>
-        <v>typedef void spi_config_num _spi(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O16," ",LOWER(F16), "_", LOWER(H16),"(", I16 ,");")</f>
+        <v>typedef void spi_config_num_spi(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2139,8 +2145,8 @@
         <v>31</v>
       </c>
       <c r="P17" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O17," ",LOWER(F17), " _", LOWER(H17),"(", I17 ,");")</f>
-        <v>typedef void spi_config_num _spi(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O17," ",LOWER(F17), "_", LOWER(H17),"(", I17 ,");")</f>
+        <v>typedef void spi_config_num_spi(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="18" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2219,8 +2225,8 @@
         <v>55</v>
       </c>
       <c r="P19" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O19," ",LOWER(F19), " _", LOWER(H19),"(", I19 ,");")</f>
-        <v>typedef int ini_num _ini(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O19," ",LOWER(F19), "_", LOWER(H19),"(", I19 ,");")</f>
+        <v>typedef int ini_num_ini(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2271,8 +2277,8 @@
         <v>55</v>
       </c>
       <c r="P20" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O20," ",LOWER(F20), " _", LOWER(H20),"(", I20 ,");")</f>
-        <v>typedef int ini_num _ini(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O20," ",LOWER(F20), "_", LOWER(H20),"(", I20 ,");")</f>
+        <v>typedef int ini_num_ini(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="21" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2351,8 +2357,8 @@
         <v>31</v>
       </c>
       <c r="P22" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O22," ",LOWER(F22), " _", LOWER(H22),"(", I22 ,");")</f>
-        <v>typedef void configure_lml_port_num _loopback(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O22," ",LOWER(F22), "_", LOWER(H22),"(", I22 ,");")</f>
+        <v>typedef void configure_lml_port_num_loopback(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="23" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2431,8 +2437,8 @@
         <v>31</v>
       </c>
       <c r="P24" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O24," ",LOWER(F24), " _", LOWER(H24),"(", I24 ,");")</f>
-        <v>typedef void one_param_const_bool_num _other(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O24," ",LOWER(F24), "_", LOWER(H24),"(", I24 ,");")</f>
+        <v>typedef void one_param_const_bool_num_other(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="68.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2483,8 +2489,8 @@
         <v>31</v>
       </c>
       <c r="P25" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O25," ",LOWER(F25), " _", LOWER(H25),"(", I25 ,");")</f>
-        <v>typedef void one_param_const_bool_num _buff(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O25," ",LOWER(F25), "_", LOWER(H25),"(", I25 ,");")</f>
+        <v>typedef void one_param_const_bool_num_buff(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="68.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2535,8 +2541,8 @@
         <v>31</v>
       </c>
       <c r="P26" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O26," ",LOWER(F26), " _", LOWER(H26),"(", I26 ,");")</f>
-        <v>typedef void one_param_const_bool_num _buff(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O26," ",LOWER(F26), "_", LOWER(H26),"(", I26 ,");")</f>
+        <v>typedef void one_param_const_bool_num_buff(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="79.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2587,8 +2593,8 @@
         <v>31</v>
       </c>
       <c r="P27" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O27," ",LOWER(F27), " _", LOWER(H27),"(", I27 ,");")</f>
-        <v>typedef void one_param_const_bool_num _other(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O27," ",LOWER(F27), "_", LOWER(H27),"(", I27 ,");")</f>
+        <v>typedef void one_param_const_bool_num_other(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="28" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2667,8 +2673,8 @@
         <v>31</v>
       </c>
       <c r="P29" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O29," ",LOWER(F29), " _", LOWER(H29),"(", I29 ,");")</f>
-        <v>typedef void one_param_lms7002m_chan_num _buff(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O29," ",LOWER(F29), "_", LOWER(H29),"(", I29 ,");")</f>
+        <v>typedef void one_param_lms7002m_chan_num_buff(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="113.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2719,8 +2725,8 @@
         <v>31</v>
       </c>
       <c r="P30" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O30," ",LOWER(F30), " _", LOWER(H30),"(", I30 ,");")</f>
-        <v>typedef void one_param_lms7002m_chan_num _mac(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O30," ",LOWER(F30), "_", LOWER(H30),"(", I30 ,");")</f>
+        <v>typedef void one_param_lms7002m_chan_num_mac(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="90.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2771,8 +2777,8 @@
         <v>31</v>
       </c>
       <c r="P31" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O31," ",LOWER(F31), " _", LOWER(H31),"(", I31 ,");")</f>
-        <v>typedef void one_param_lms7002m_chan_num _mac(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O31," ",LOWER(F31), "_", LOWER(H31),"(", I31 ,");")</f>
+        <v>typedef void one_param_lms7002m_chan_num_mac(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="57.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2823,8 +2829,8 @@
         <v>31</v>
       </c>
       <c r="P32" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O32," ",LOWER(F32), " _", LOWER(H32),"(", I32 ,");")</f>
-        <v>typedef void one_param_lms7002m_chan_num _enable channel(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O32," ",LOWER(F32), "_", LOWER(H32),"(", I32 ,");")</f>
+        <v>typedef void one_param_lms7002m_chan_num_enable channel(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2875,8 +2881,8 @@
         <v>31</v>
       </c>
       <c r="P33" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O33," ",LOWER(F33), " _", LOWER(H33),"(", I33 ,");")</f>
-        <v>typedef void one_param_lms7002m_chan_num _enable channel(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O33," ",LOWER(F33), "_", LOWER(H33),"(", I33 ,");")</f>
+        <v>typedef void one_param_lms7002m_chan_num_enable channel(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2924,8 +2930,8 @@
         <v>55</v>
       </c>
       <c r="P34" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O34," ",LOWER(F34), " _", LOWER(H34),"(", I34 ,");")</f>
-        <v>typedef int one_param_lms7002m_chan_num _enable channel(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O34," ",LOWER(F34), "_", LOWER(H34),"(", I34 ,");")</f>
+        <v>typedef int one_param_lms7002m_chan_num_enable channel(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2973,8 +2979,8 @@
         <v>55</v>
       </c>
       <c r="P35" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O35," ",LOWER(F35), " _", LOWER(H35),"(", I35 ,");")</f>
-        <v>typedef int one_param_lms7002m_chan_num _enable channel(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O35," ",LOWER(F35), "_", LOWER(H35),"(", I35 ,");")</f>
+        <v>typedef int one_param_lms7002m_chan_num_enable channel(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="36" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3053,8 +3059,8 @@
         <v>31</v>
       </c>
       <c r="P37" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O37," ",LOWER(F37), " _", LOWER(H37),"(", I37 ,");")</f>
-        <v>typedef void two_param_lms7002m_dir_int_num _iq(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O37," ",LOWER(F37), "_", LOWER(H37),"(", I37 ,");")</f>
+        <v>typedef void two_param_lms7002m_dir_int_num_iq(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="38" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3133,8 +3139,8 @@
         <v>31</v>
       </c>
       <c r="P39" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O39," ",LOWER(F39), " _", LOWER(H39),"(", I39 ,");")</f>
-        <v>typedef void ldo_enable_num _enable(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O39," ",LOWER(F39), "_", LOWER(H39),"(", I39 ,");")</f>
+        <v>typedef void ldo_enable_num_enable(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="40" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3213,8 +3219,8 @@
         <v>31</v>
       </c>
       <c r="P41" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O41," ",LOWER(F41), " _", LOWER(H41),"(", I41 ,");")</f>
-        <v>typedef void afe_enable_num _enable(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O41," ",LOWER(F41), "_", LOWER(H41),"(", I41 ,");")</f>
+        <v>typedef void afe_enable_num_enable(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="42" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3293,8 +3299,8 @@
         <v>55</v>
       </c>
       <c r="P43" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O43," ",LOWER(F43), " _", LOWER(H43),"(", I43 ,");")</f>
-        <v>typedef int set_data_clock_num _sampling(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O43," ",LOWER(F43), "_", LOWER(H43),"(", I43 ,");")</f>
+        <v>typedef int set_data_clock_num_sampling(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="44" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3373,8 +3379,8 @@
         <v>31</v>
       </c>
       <c r="P45" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O45," ",LOWER(F45), " _", LOWER(H45),"(", I45 ,");")</f>
-        <v>typedef void set_nco_freq_num _frequency tunning(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O45," ",LOWER(F45), "_", LOWER(H45),"(", I45 ,");")</f>
+        <v>typedef void set_nco_freq_num_frequency tunning(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="46" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3453,8 +3459,8 @@
         <v>55</v>
       </c>
       <c r="P47" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O47," ",LOWER(F47), " _", LOWER(H47),"(", I47 ,");")</f>
-        <v>typedef int set_gfir_taps_num _fir(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O47," ",LOWER(F47), "_", LOWER(H47),"(", I47 ,");")</f>
+        <v>typedef int set_gfir_taps_num_fir(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="48" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3533,8 +3539,8 @@
         <v>55</v>
       </c>
       <c r="P49" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O49," ",LOWER(F49), " _", LOWER(H49),"(", I49 ,");")</f>
-        <v>typedef int set_lo_freq_num _frequency tunning(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O49," ",LOWER(F49), "_", LOWER(H49),"(", I49 ,");")</f>
+        <v>typedef int set_lo_freq_num_frequency tunning(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="50" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3613,8 +3619,8 @@
         <v>31</v>
       </c>
       <c r="P51" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O51," ",LOWER(F51), " _", LOWER(H51),"(", I51 ,");")</f>
-        <v>typedef void two_param_lms_const_bool_num _enable(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O51," ",LOWER(F51), "_", LOWER(H51),"(", I51 ,");")</f>
+        <v>typedef void two_param_lms_const_bool_num_enable(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="79.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3665,8 +3671,8 @@
         <v>31</v>
       </c>
       <c r="P52" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O52," ",LOWER(F52), " _", LOWER(H52),"(", I52 ,");")</f>
-        <v>typedef void two_param_lms_const_bool_num _enable(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O52," ",LOWER(F52), "_", LOWER(H52),"(", I52 ,");")</f>
+        <v>typedef void two_param_lms_const_bool_num_enable(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3717,8 +3723,8 @@
         <v>31</v>
       </c>
       <c r="P53" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O53," ",LOWER(F53), " _", LOWER(H53),"(", I53 ,");")</f>
-        <v>typedef void two_param_lms_const_bool_num _enable(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O53," ",LOWER(F53), "_", LOWER(H53),"(", I53 ,");")</f>
+        <v>typedef void two_param_lms_const_bool_num_enable(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3769,8 +3775,8 @@
         <v>31</v>
       </c>
       <c r="P54" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O54," ",LOWER(F54), " _", LOWER(H54),"(", I54 ,");")</f>
-        <v>typedef void two_param_lms_const_bool_num _enable(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O54," ",LOWER(F54), "_", LOWER(H54),"(", I54 ,");")</f>
+        <v>typedef void two_param_lms_const_bool_num_enable(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3821,8 +3827,8 @@
         <v>31</v>
       </c>
       <c r="P55" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O55," ",LOWER(F55), " _", LOWER(H55),"(", I55 ,");")</f>
-        <v>typedef void two_param_lms_const_bool_num _enable(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O55," ",LOWER(F55), "_", LOWER(H55),"(", I55 ,");")</f>
+        <v>typedef void two_param_lms_const_bool_num_enable(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3873,8 +3879,8 @@
         <v>31</v>
       </c>
       <c r="P56" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O56," ",LOWER(F56), " _", LOWER(H56),"(", I56 ,");")</f>
-        <v>typedef void two_param_lms_const_bool_num _enable(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O56," ",LOWER(F56), "_", LOWER(H56),"(", I56 ,");")</f>
+        <v>typedef void two_param_lms_const_bool_num_enable(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3925,8 +3931,8 @@
         <v>31</v>
       </c>
       <c r="P57" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O57," ",LOWER(F57), " _", LOWER(H57),"(", I57 ,");")</f>
-        <v>typedef void two_param_lms_const_bool_num _enable(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O57," ",LOWER(F57), "_", LOWER(H57),"(", I57 ,");")</f>
+        <v>typedef void two_param_lms_const_bool_num_enable(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="68.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3977,8 +3983,8 @@
         <v>31</v>
       </c>
       <c r="P58" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O58," ",LOWER(F58), " _", LOWER(H58),"(", I58 ,");")</f>
-        <v>typedef void two_param_lms_const_bool_num _test(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O58," ",LOWER(F58), "_", LOWER(H58),"(", I58 ,");")</f>
+        <v>typedef void two_param_lms_const_bool_num_test(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4029,8 +4035,8 @@
         <v>31</v>
       </c>
       <c r="P59" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O59," ",LOWER(F59), " _", LOWER(H59),"(", I59 ,");")</f>
-        <v>typedef void two_param_lms_const_bool_num _enable(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O59," ",LOWER(F59), "_", LOWER(H59),"(", I59 ,");")</f>
+        <v>typedef void two_param_lms_const_bool_num_enable(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="60" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4109,8 +4115,8 @@
         <v>31</v>
       </c>
       <c r="P61" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O61," ",LOWER(F61), " _", LOWER(H61),"(", I61 ,");")</f>
-        <v>typedef void two_param_chant_sizet_num _sampling(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O61," ",LOWER(F61), "_", LOWER(H61),"(", I61 ,");")</f>
+        <v>typedef void two_param_chant_sizet_num_sampling(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4161,8 +4167,8 @@
         <v>31</v>
       </c>
       <c r="P62" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O62," ",LOWER(F62), " _", LOWER(H62),"(", I62 ,");")</f>
-        <v>typedef void two_param_chant_sizet_num _sampling(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O62," ",LOWER(F62), "_", LOWER(H62),"(", I62 ,");")</f>
+        <v>typedef void two_param_chant_sizet_num_sampling(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="63" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4241,8 +4247,8 @@
         <v>31</v>
       </c>
       <c r="P64" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O64," ",LOWER(F64), " _", LOWER(H64),"(", I64 ,");")</f>
-        <v>typedef void sp_tsg_num _iq(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O64," ",LOWER(F64), "_", LOWER(H64),"(", I64 ,");")</f>
+        <v>typedef void sp_tsg_num_iq(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="57.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4293,8 +4299,8 @@
         <v>31</v>
       </c>
       <c r="P65" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O65," ",LOWER(F65), " _", LOWER(H65),"(", I65 ,");")</f>
-        <v>typedef void sp_tsg_num _iq(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O65," ",LOWER(F65), "_", LOWER(H65),"(", I65 ,");")</f>
+        <v>typedef void sp_tsg_num_iq(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="66" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4373,8 +4379,8 @@
         <v>31</v>
       </c>
       <c r="P67" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O67," ",LOWER(F67), " _", LOWER(H67),"(", I67 ,");")</f>
-        <v>typedef void txstp_correction_num _calibrate(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O67," ",LOWER(F67), "_", LOWER(H67),"(", I67 ,");")</f>
+        <v>typedef void txstp_correction_num_calibrate(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="146.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4425,8 +4431,8 @@
         <v>31</v>
       </c>
       <c r="P68" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O68," ",LOWER(F68), " _", LOWER(H68),"(", I68 ,");")</f>
-        <v>typedef void txstp_correction_num _calibrate(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O68," ",LOWER(F68), "_", LOWER(H68),"(", I68 ,");")</f>
+        <v>typedef void txstp_correction_num_calibrate(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="69" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4505,8 +4511,8 @@
         <v>31</v>
       </c>
       <c r="P70" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O70," ",LOWER(F70), " _", LOWER(H70),"(", I70 ,");")</f>
-        <v>typedef void rxtsp_num _calibrate(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O70," ",LOWER(F70), "_", LOWER(H70),"(", I70 ,");")</f>
+        <v>typedef void rxtsp_num_calibrate(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="153.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4557,8 +4563,8 @@
         <v>31</v>
       </c>
       <c r="P71" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O71," ",LOWER(F71), " _", LOWER(H71),"(", I71 ,");")</f>
-        <v>typedef void rxtsp_num _calibrate(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O71," ",LOWER(F71), "_", LOWER(H71),"(", I71 ,");")</f>
+        <v>typedef void rxtsp_num_calibrate(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="72" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4637,8 +4643,8 @@
         <v>31</v>
       </c>
       <c r="P73" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O73," ",LOWER(F73), " _", LOWER(H73),"(", I73 ,");")</f>
-        <v>typedef void set_path_and_band_num _band(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O73," ",LOWER(F73), "_", LOWER(H73),"(", I73 ,");")</f>
+        <v>typedef void set_path_and_band_num_band(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="68.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4689,8 +4695,8 @@
         <v>31</v>
       </c>
       <c r="P74" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O74," ",LOWER(F74), " _", LOWER(H74),"(", I74 ,");")</f>
-        <v>typedef void set_path_and_band_num _test(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O74," ",LOWER(F74), "_", LOWER(H74),"(", I74 ,");")</f>
+        <v>typedef void set_path_and_band_num_test(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4741,8 +4747,8 @@
         <v>31</v>
       </c>
       <c r="P75" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O75," ",LOWER(F75), " _", LOWER(H75),"(", I75 ,");")</f>
-        <v>typedef void set_path_and_band_num _band(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O75," ",LOWER(F75), "_", LOWER(H75),"(", I75 ,");")</f>
+        <v>typedef void set_path_and_band_num_band(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="79.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4793,8 +4799,8 @@
         <v>31</v>
       </c>
       <c r="P76" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O76," ",LOWER(F76), " _", LOWER(H76),"(", I76 ,");")</f>
-        <v>typedef void set_path_and_band_num _band(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O76," ",LOWER(F76), "_", LOWER(H76),"(", I76 ,");")</f>
+        <v>typedef void set_path_and_band_num_band(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="45.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4845,8 +4851,8 @@
         <v>31</v>
       </c>
       <c r="P77" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O77," ",LOWER(F77), " _", LOWER(H77),"(", I77 ,");")</f>
-        <v>typedef void set_path_and_band_num _enable channel(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O77," ",LOWER(F77), "_", LOWER(H77),"(", I77 ,");")</f>
+        <v>typedef void set_path_and_band_num_enable channel(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="78" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4925,8 +4931,8 @@
         <v>31</v>
       </c>
       <c r="P79" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O79," ",LOWER(F79), " _", LOWER(H79),"(", I79 ,");")</f>
-        <v>typedef void tbb_loop_back_enable_num _iq(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O79," ",LOWER(F79), "_", LOWER(H79),"(", I79 ,");")</f>
+        <v>typedef void tbb_loop_back_enable_num_iq(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="80" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5005,8 +5011,8 @@
         <v>55</v>
       </c>
       <c r="P81" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O81," ",LOWER(F81), " _", LOWER(H81),"(", I81 ,");")</f>
-        <v>typedef int bb_filer_set_num _calibrate(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O81," ",LOWER(F81), "_", LOWER(H81),"(", I81 ,");")</f>
+        <v>typedef int bb_filer_set_num_calibrate(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="57.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5057,8 +5063,8 @@
         <v>55</v>
       </c>
       <c r="P82" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O82," ",LOWER(F82), " _", LOWER(H82),"(", I82 ,");")</f>
-        <v>typedef int bb_filer_set_num _calibrate(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O82," ",LOWER(F82), "_", LOWER(H82),"(", I82 ,");")</f>
+        <v>typedef int bb_filer_set_num_calibrate(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="83" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5137,8 +5143,8 @@
         <v>31</v>
       </c>
       <c r="P84" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O84," ",LOWER(F84), " _", LOWER(H84),"(", I84 ,");")</f>
-        <v>typedef void trf_rbb_rfe_num _frequency tunning(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O84," ",LOWER(F84), "_", LOWER(H84),"(", I84 ,");")</f>
+        <v>typedef void trf_rbb_rfe_num_frequency tunning(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="45.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5189,8 +5195,8 @@
         <v>31</v>
       </c>
       <c r="P85" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O85," ",LOWER(F85), " _", LOWER(H85),"(", I85 ,");")</f>
-        <v>typedef void trf_rbb_rfe_num _frequency tunning(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O85," ",LOWER(F85), "_", LOWER(H85),"(", I85 ,");")</f>
+        <v>typedef void trf_rbb_rfe_num_frequency tunning(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5241,8 +5247,8 @@
         <v>221</v>
       </c>
       <c r="P86" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O86," ",LOWER(F86), " _", LOWER(H86),"(", I86 ,");")</f>
-        <v>typedef double trf_rbb_rfe_num _gain(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O86," ",LOWER(F86), "_", LOWER(H86),"(", I86 ,");")</f>
+        <v>typedef double trf_rbb_rfe_num_gain(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="45.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5293,8 +5299,8 @@
         <v>221</v>
       </c>
       <c r="P87" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O87," ",LOWER(F87), " _", LOWER(H87),"(", I87 ,");")</f>
-        <v>typedef double trf_rbb_rfe_num _gain(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O87," ",LOWER(F87), "_", LOWER(H87),"(", I87 ,");")</f>
+        <v>typedef double trf_rbb_rfe_num_gain(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5345,8 +5351,8 @@
         <v>221</v>
       </c>
       <c r="P88" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O88," ",LOWER(F88), " _", LOWER(H88),"(", I88 ,");")</f>
-        <v>typedef double trf_rbb_rfe_num _gain(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O88," ",LOWER(F88), "_", LOWER(H88),"(", I88 ,");")</f>
+        <v>typedef double trf_rbb_rfe_num_gain(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5397,8 +5403,8 @@
         <v>221</v>
       </c>
       <c r="P89" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O89," ",LOWER(F89), " _", LOWER(H89),"(", I89 ,");")</f>
-        <v>typedef double trf_rbb_rfe_num _gain(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O89," ",LOWER(F89), "_", LOWER(H89),"(", I89 ,");")</f>
+        <v>typedef double trf_rbb_rfe_num_gain(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="45.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5449,8 +5455,8 @@
         <v>221</v>
       </c>
       <c r="P90" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O90," ",LOWER(F90), " _", LOWER(H90),"(", I90 ,");")</f>
-        <v>typedef double trf_rbb_rfe_num _gain(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O90," ",LOWER(F90), "_", LOWER(H90),"(", I90 ,");")</f>
+        <v>typedef double trf_rbb_rfe_num_gain(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5501,8 +5507,8 @@
         <v>221</v>
       </c>
       <c r="P91" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O91," ",LOWER(F91), " _", LOWER(H91),"(", I91 ,");")</f>
-        <v>typedef double trf_rbb_rfe_num _gain(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O91," ",LOWER(F91), "_", LOWER(H91),"(", I91 ,");")</f>
+        <v>typedef double trf_rbb_rfe_num_gain(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="92" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5581,8 +5587,8 @@
         <v>237</v>
       </c>
       <c r="P93" s="2" t="str">
-        <f aca="false">CONCATENATE("typedef ",O93," ",LOWER(F93), " _", LOWER(H93),"(", I93 ,");")</f>
-        <v>typedef uint16_t readrssi_num _rssi(LMS7002M_t *);</v>
+        <f aca="false">CONCATENATE("typedef ",O93," ",LOWER(F93), "_", LOWER(H93),"(", I93 ,");")</f>
+        <v>typedef uint16_t readrssi_num_rssi(LMS7002M_t *);</v>
       </c>
     </row>
     <row r="94" s="10" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>